<commit_message>
Update XLSX test file for create peptide ordering form test
</commit_message>
<xml_diff>
--- a/tests/test_data/pvacseq_create_peptide_ordering_form/expected_output.Colored_Peptides.xlsx
+++ b/tests/test_data/pvacseq_create_peptide_ordering_form/expected_output.Colored_Peptides.xlsx
@@ -3750,6 +3750,16 @@
         <scheme val="minor"/>
       </rPr>
       <t>P</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
     </r>
   </si>
   <si>
@@ -6426,7 +6436,7 @@
         <v>42</v>
       </c>
       <c r="E8">
-        <v>4608.668</v>
+        <v>4711.810899999999</v>
       </c>
       <c r="F8" t="s">
         <v>23</v>

</xml_diff>